<commit_message>
Data and code updation.
</commit_message>
<xml_diff>
--- a/12612645.xlsx
+++ b/12612645.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shash\Desktop\MinorProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C7F77C2-62ED-4967-B2A1-A5890CBE0E32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56295DFD-46B9-4421-AA72-5A62DC325B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="71">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2279,180 +2279,356 @@
       </c>
       <c r="N33" s="17"/>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+    <row r="34" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="8">
+        <v>46279</v>
+      </c>
+      <c r="B34" s="14">
+        <v>300</v>
+      </c>
+      <c r="C34" s="14">
+        <v>0</v>
+      </c>
+      <c r="D34" s="14">
+        <v>180</v>
+      </c>
+      <c r="E34" s="14">
+        <v>90</v>
+      </c>
+      <c r="F34" s="14">
+        <v>200</v>
+      </c>
+      <c r="G34" s="14">
+        <v>4</v>
+      </c>
+      <c r="H34" s="14">
+        <v>300</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
+        <v>370</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N34" s="17"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+      <c r="A35" s="8">
+        <v>46280</v>
+      </c>
+      <c r="B35" s="14">
+        <v>240</v>
+      </c>
+      <c r="C35" s="14">
+        <v>0</v>
+      </c>
+      <c r="D35" s="14">
+        <v>240</v>
+      </c>
+      <c r="E35" s="14">
+        <v>60</v>
+      </c>
+      <c r="F35" s="14">
+        <v>350</v>
+      </c>
+      <c r="G35" s="14">
+        <v>7</v>
+      </c>
+      <c r="H35" s="14">
+        <v>240</v>
+      </c>
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>1130</v>
+      </c>
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
+        <v>310</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="N35" s="17"/>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+      <c r="A36" s="8">
+        <v>46281</v>
+      </c>
+      <c r="B36" s="14">
+        <v>180</v>
+      </c>
+      <c r="C36" s="14">
+        <v>0</v>
+      </c>
+      <c r="D36" s="14">
+        <v>180</v>
+      </c>
+      <c r="E36" s="14">
+        <v>120</v>
+      </c>
+      <c r="F36" s="14">
+        <v>350</v>
+      </c>
+      <c r="G36" s="14">
+        <v>7</v>
+      </c>
+      <c r="H36" s="14">
+        <v>270</v>
+      </c>
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
+        <v>340</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="N36" s="17"/>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+    <row r="37" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="8">
+        <v>46282</v>
+      </c>
+      <c r="B37" s="14">
+        <v>300</v>
+      </c>
+      <c r="C37" s="14">
+        <v>0</v>
+      </c>
+      <c r="D37" s="14">
+        <v>180</v>
+      </c>
+      <c r="E37" s="14">
+        <v>90</v>
+      </c>
+      <c r="F37" s="14">
+        <v>200</v>
+      </c>
+      <c r="G37" s="14">
+        <v>4</v>
+      </c>
+      <c r="H37" s="14">
+        <v>180</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
+        <v>490</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N37" s="17"/>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+    <row r="38" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="8">
+        <v>46283</v>
+      </c>
+      <c r="B38" s="14">
+        <v>240</v>
+      </c>
+      <c r="C38" s="14">
+        <v>0</v>
+      </c>
+      <c r="D38" s="14">
+        <v>240</v>
+      </c>
+      <c r="E38" s="14">
+        <v>120</v>
+      </c>
+      <c r="F38" s="14">
+        <v>250</v>
+      </c>
+      <c r="G38" s="14">
+        <v>5</v>
+      </c>
+      <c r="H38" s="14">
+        <v>180</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>1030</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
+        <v>410</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N38" s="17"/>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+    <row r="39" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="8">
+        <v>46284</v>
+      </c>
+      <c r="B39" s="14">
+        <v>360</v>
+      </c>
+      <c r="C39" s="14">
+        <v>0</v>
+      </c>
+      <c r="D39" s="14">
+        <v>240</v>
+      </c>
+      <c r="E39" s="14">
+        <v>180</v>
+      </c>
+      <c r="F39" s="14">
+        <v>0</v>
+      </c>
+      <c r="G39" s="14">
+        <v>0</v>
+      </c>
+      <c r="H39" s="14">
+        <v>210</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>990</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
+        <v>450</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N39" s="17"/>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+    <row r="40" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="8">
+        <v>46285</v>
+      </c>
+      <c r="B40" s="14">
+        <v>300</v>
+      </c>
+      <c r="C40" s="14">
+        <v>0</v>
+      </c>
+      <c r="D40" s="14">
+        <v>300</v>
+      </c>
+      <c r="E40" s="14">
+        <v>90</v>
+      </c>
+      <c r="F40" s="14">
+        <v>0</v>
+      </c>
+      <c r="G40" s="14">
+        <v>0</v>
+      </c>
+      <c r="H40" s="14">
+        <v>240</v>
+      </c>
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>930</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
+        <v>510</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N40" s="17"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="13"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+      <c r="A41" s="8">
+        <v>46286</v>
+      </c>
+      <c r="B41" s="14">
+        <v>240</v>
+      </c>
+      <c r="C41" s="14">
+        <v>0</v>
+      </c>
+      <c r="D41" s="14">
+        <v>240</v>
+      </c>
+      <c r="E41" s="14">
+        <v>90</v>
+      </c>
+      <c r="F41" s="14">
+        <v>200</v>
+      </c>
+      <c r="G41" s="14">
+        <v>4</v>
+      </c>
+      <c r="H41" s="14">
+        <v>210</v>
+      </c>
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>980</v>
+      </c>
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
+        <v>460</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N41" s="17"/>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
@@ -10405,5 +10581,8 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <ignoredErrors>
+    <ignoredError sqref="I34:I41" formulaRange="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>